<commit_message>
Refine BOR outputs and add CI model validation
</commit_message>
<xml_diff>
--- a/LNG_BOR_Model.xlsx
+++ b/LNG_BOR_Model.xlsx
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>압력↑→비등점↑→BOG↓ (근사, 최소 0.8)</t>
+          <t>단순 선형 근사(최소 0.8), 정밀 계산은 Antoine 식 기반 고도화 가능</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>BOG 일일 증발량 [kg/day]</t>
+          <t>BOG 일일 증발량 (중간계산) [kg/day]</t>
         </is>
       </c>
       <c r="B38" s="12">
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="D38" s="4">
-        <f> BOG유량 × 86400 × 압력보정</f>
+        <f> BOG유량 × 86400 × 압력보정 (중간계산값)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel formula errors: rename sheet tabs to ASCII (Input/PropertyDB/BOR_Calc/Measure)
</commit_message>
<xml_diff>
--- a/LNG_BOR_Model.xlsx
+++ b/LNG_BOR_Model.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_입력조건" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_물성DB" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_BOR계산" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_계측보정" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Input" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PropertyDB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BOR_Calc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Measure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>'1_입력조건'!B4/2</f>
+        <f>Input!B4/2</f>
         <v/>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>2*PI()*B4*'1_입력조건'!B5</f>
+        <f>2*PI()*B4*Input!B5</f>
         <v/>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>PI()*B4^2*'1_입력조건'!B5+(4/3)*PI()*B4^3</f>
+        <f>PI()*B4^2*Input!B5+(4/3)*PI()*B4^3</f>
         <v/>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>B8*'1_입력조건'!B6/100</f>
+        <f>B8*Input!B6/100</f>
         <v/>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>VLOOKUP('1_입력조건'!B11,'2_물성DB'!A4:B9,2,FALSE)</f>
+        <f>VLOOKUP(Input!B11,PropertyDB!A4:B9,2,FALSE)</f>
         <v/>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>IF('1_입력조건'!B13&lt;10,0.7,IF('1_입력조건'!B13&lt;100,0.85,1.0))</f>
+        <f>IF(Input!B13&lt;10,0.7,IF(Input!B13&lt;100,0.85,1.0))</f>
         <v/>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>'1_입력조건'!B12/(B13*B7)</f>
+        <f>Input!B12/(B13*B7)</f>
         <v/>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>VLOOKUP('1_입력조건'!B22,'2_물성DB'!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>VLOOKUP('1_입력조건'!B23,'2_물성DB'!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>VLOOKUP('1_입력조건'!B24,'2_물성DB'!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>(B16*'1_입력조건'!C22+B17*'1_입력조건'!C23+B18*'1_입력조건'!C24)/('1_입력조건'!C22+'1_입력조건'!C23+'1_입력조건'!C24)</f>
+        <f>(B16*Input!C22+B17*Input!C23+B18*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
         <v/>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>VLOOKUP('1_입력조건'!B22,'2_물성DB'!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>VLOOKUP('1_입력조건'!B23,'2_물성DB'!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>VLOOKUP('1_입력조건'!B24,'2_물성DB'!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>(B20*'1_입력조건'!C22+B21*'1_입력조건'!C23+B22*'1_입력조건'!C24)/('1_입력조건'!C22+'1_입력조건'!C23+'1_입력조건'!C24)</f>
+        <f>(B20*Input!C22+B21*Input!C23+B22*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
         <v/>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>VLOOKUP('1_입력조건'!B22,'2_물성DB'!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>VLOOKUP('1_입력조건'!B23,'2_물성DB'!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>VLOOKUP('1_입력조건'!B24,'2_물성DB'!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1760,7 +1760,7 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>(B24*'1_입력조건'!C22+B25*'1_입력조건'!C23+B26*'1_입력조건'!C24)/('1_입력조건'!C22+'1_입력조건'!C23+'1_입력조건'!C24)</f>
+        <f>(B24*Input!C22+B25*Input!C23+B26*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
         <v/>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1788,7 +1788,7 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>MAX(0.8,1-(('1_입력조건'!B8-1.013)*0.05))</f>
+        <f>MAX(0.8,1-((Input!B8-1.013)*0.05))</f>
         <v/>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>'1_입력조건'!B9-B27</f>
+        <f>Input!B9-B27</f>
         <v/>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>VLOOKUP('1_입력조건'!B15,'2_물성DB'!A22:B24,2,FALSE)</f>
+        <f>VLOOKUP(Input!B15,PropertyDB!A22:B24,2,FALSE)</f>
         <v/>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>B32*('1_입력조건'!B16/100)*B33</f>
+        <f>B32*(Input!B16/100)*B33</f>
         <v/>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>'1_입력조건'!B19</f>
+        <f>Input!B19</f>
         <v/>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>IF('1_입력조건'!B18&lt;6,1.15,IF('1_입력조건'!B18&lt;12,1.05,1.0))</f>
+        <f>IF(Input!B18&lt;6,1.15,IF(Input!B18&lt;12,1.05,1.0))</f>
         <v/>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>'3_BOR계산'!B39</f>
+        <f>BOR_Calc!B39</f>
         <v/>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="B13" s="13">
-        <f>'3_BOR계산'!B40</f>
+        <f>BOR_Calc!B40</f>
         <v/>
       </c>
       <c r="C13" s="4" t="inlineStr">

</xml_diff>

<commit_message>
fix BOR_Calc composition formulas and validation
</commit_message>
<xml_diff>
--- a/LNG_BOR_Model.xlsx
+++ b/LNG_BOR_Model.xlsx
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,3,FALSE)</f>
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>(B16*Input!C22+B17*Input!C23+B18*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
+        <f>(B16*Input!B22+B17*Input!B23+B18*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
         <v/>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,4,FALSE)</f>
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>(B20*Input!C22+B21*Input!C23+B22*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
+        <f>(B20*Input!B22+B21*Input!B23+B22*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
         <v/>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>VLOOKUP(Input!B22,PropertyDB!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>VLOOKUP(Input!B23,PropertyDB!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>VLOOKUP(Input!B24,PropertyDB!A13:E18,5,FALSE)</f>
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1760,7 +1760,7 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>(B24*Input!C22+B25*Input!C23+B26*Input!C24)/(Input!C22+Input!C23+Input!C24)</f>
+        <f>(B24*Input!B22+B25*Input!B23+B26*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
         <v/>
       </c>
       <c r="C27" s="4" t="inlineStr">

</xml_diff>

<commit_message>
fix: update Input layout, notes, and validation for BOR workbook
</commit_message>
<xml_diff>
--- a/LNG_BOR_Model.xlsx
+++ b/LNG_BOR_Model.xlsx
@@ -68,7 +68,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -92,12 +92,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00B4C6E7"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -146,7 +151,18 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -164,16 +180,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -541,13 +554,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -585,6 +605,11 @@
           <t>▶ 탱크 기하 조건</t>
         </is>
       </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>▶ 탱크 형상(고정) 및 사양 정보</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -621,6 +646,15 @@
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>원통형 LNG 탱크 (고정)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -641,314 +675,648 @@
           <t>0~100</t>
         </is>
       </c>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>▶ 운전 조건</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>탱크 내부 체적 [m³]</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>PI()*(B4/2)^2*B5+(4/3)*PI()*(B4/2)^3</f>
+        <v/>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>내경·길이로 자동 계산</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="8" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>LNG 체적 [m³]</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>B7*B6/100</f>
+        <v/>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>체적 × 충전율</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>▶ 운전 조건</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>탱크 내부 압력 [bar(a)]</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B10" s="5" t="n">
         <v>1.13</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>bar(a)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>절대압</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>외부(주위) 온도 [℃]</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>℃</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>▶ 단열재 조건</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>단열재 종류</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Perlite(진공)</t>
-        </is>
+          <t>외부(주위) 온도 [℃]</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>25</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>드롭다운 선택</t>
+          <t>℃</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>■ 사양 패널 (셀 연동)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>단열재 두께 [m]</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>▶ 단열재 조건</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>탱크 내경</t>
+        </is>
+      </c>
+      <c r="G12" s="10">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>진공도 [Pa]</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>1</v>
+          <t>단열재 종류</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Perlite(진공)</t>
+        </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>진공단열 시 적용</t>
+          <t>드롭다운 선택</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>탱크 길이</t>
+        </is>
+      </c>
+      <c r="G13" s="10">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>▶ 배관 조건</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>단열재 두께 [m]</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>충전율</t>
+        </is>
+      </c>
+      <c r="G14" s="10">
+        <f>B6</f>
+        <v/>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>진공도 [Pa]</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>진공단열 시 적용</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>탱크 내부 체적</t>
+        </is>
+      </c>
+      <c r="G15" s="10">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>▶ 배관 조건</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>LNG 체적</t>
+        </is>
+      </c>
+      <c r="G16" s="10">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>배관 보냉/진공 여부</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>진공배관</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>드롭다운 선택</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>배관 추가 열유입 비율 [%]</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>탱크 열유입 대비</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>▶ 계측 조건</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>내부 압력</t>
+        </is>
+      </c>
+      <c r="G17" s="10">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>bar(a)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>배관 추가 열유입 비율 [%]</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>탱크 열유입 대비</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>외부 온도</t>
+        </is>
+      </c>
+      <c r="G18" s="10">
+        <f>B11</f>
+        <v/>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>℃</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>▶ 계측 조건</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>단열재 종류</t>
+        </is>
+      </c>
+      <c r="G19" s="10">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>안정화 시간 [h]</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>BOG 안정화 대기 시간</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>단열재 두께</t>
+        </is>
+      </c>
+      <c r="G20" s="10">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>BOG 계측 시간 [h]</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>실측 수집 시간</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>진공도</t>
+        </is>
+      </c>
+      <c r="G21" s="10">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>▶ LNG 조성 (상위 3성분)</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>배관 보냉/진공</t>
+        </is>
+      </c>
+      <c r="G22" s="10">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>성분 이름</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>몰분율 [mol%]</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>mol%</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>주성분</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Ethane</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>mol%</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>배관 열유입 비율</t>
+        </is>
+      </c>
+      <c r="G23" s="10">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>mol%</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>주성분</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>성분1 이름</t>
+        </is>
+      </c>
+      <c r="G24" s="10">
+        <f>A24</f>
+        <v/>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Ethane</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>mol%</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>성분1 몰분율</t>
+        </is>
+      </c>
+      <c r="G25" s="10">
+        <f>B24</f>
+        <v/>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>mol%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>Propane</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>mol%</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>합계 100%</t>
         </is>
       </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>성분2 이름</t>
+        </is>
+      </c>
+      <c r="G26" s="10">
+        <f>A25</f>
+        <v/>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>성분2 몰분율</t>
+        </is>
+      </c>
+      <c r="G27" s="10">
+        <f>B25</f>
+        <v/>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>mol%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>성분3 이름</t>
+        </is>
+      </c>
+      <c r="G28" s="10">
+        <f>A26</f>
+        <v/>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>성분3 몰분율</t>
+        </is>
+      </c>
+      <c r="G29" s="10">
+        <f>B26</f>
+        <v/>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>mol%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="F3:L3"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="G5:K9"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
       <formula1>"Polyurethane Foam (PUF),Perlite(대기압),Perlite(진공),MLI(다층진공단열),Glass Wool,Vacuum Panel"</formula1>
     </dataValidation>
-    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
       <formula1>"보냉없음,일반보냉,진공배관"</formula1>
     </dataValidation>
-    <dataValidation sqref="B22:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
+    <dataValidation sqref="B24:B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
       <formula1>"Methane,Ethane,Propane,Nitrogen,i-Butane,n-Butane"</formula1>
     </dataValidation>
   </dataValidations>
@@ -974,7 +1342,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>LNG BOR 예측 모델 — 물성 데이터베이스 (2_물성DB)</t>
         </is>
@@ -988,74 +1356,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>단열재 종류</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>열전도율 k [W/m·K]</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Polyurethane Foam (PUF)</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="14" t="n">
         <v>0.025</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Perlite(대기압)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="14" t="n">
         <v>0.04</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Perlite(진공)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="14" t="n">
         <v>0.0015</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>MLI(다층진공단열)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="14" t="n">
         <v>0.0005</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Glass Wool</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="14" t="n">
         <v>0.038</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Vacuum Panel</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="14" t="n">
         <v>0.008</v>
       </c>
     </row>
@@ -1067,164 +1435,164 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>분자량
 [g/mol]</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>잠열 ΔHvap
 [kJ/kg]</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>액밀도
 [kg/m³]</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>비등점
 [℃]</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Methane</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="16" t="n">
         <v>16.04</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="16" t="n">
         <v>511</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="16" t="n">
         <v>422.6</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="16" t="n">
         <v>-161.5</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>주성분</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Ethane</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="16" t="n">
         <v>30.07</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="16" t="n">
         <v>489</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="16" t="n">
         <v>544.1</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="16" t="n">
         <v>-88.59999999999999</v>
       </c>
-      <c r="F14" s="11" t="inlineStr"/>
+      <c r="F14" s="16" t="inlineStr"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Propane</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="16" t="n">
         <v>44.1</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="16" t="n">
         <v>426</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="16" t="n">
         <v>581</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="16" t="n">
         <v>-42.1</v>
       </c>
-      <c r="F15" s="11" t="inlineStr"/>
+      <c r="F15" s="16" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Nitrogen</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="16" t="n">
         <v>28.01</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="16" t="n">
         <v>199</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="16" t="n">
         <v>806.6</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="16" t="n">
         <v>-195.8</v>
       </c>
-      <c r="F16" s="11" t="inlineStr"/>
+      <c r="F16" s="16" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>i-Butane</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="16" t="n">
         <v>58.12</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="16" t="n">
         <v>366</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="16" t="n">
         <v>593.4</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="16" t="n">
         <v>-11.7</v>
       </c>
-      <c r="F17" s="11" t="inlineStr"/>
+      <c r="F17" s="16" t="inlineStr"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>n-Butane</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="16" t="n">
         <v>58.12</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="16" t="n">
         <v>385</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="16" t="n">
         <v>601.8</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="16" t="n">
         <v>-0.5</v>
       </c>
-      <c r="F18" s="11" t="inlineStr"/>
+      <c r="F18" s="16" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1234,44 +1602,44 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>배관 상태</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>열유입 계수</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>보냉없음</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>일반보냉</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="16" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>진공배관</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="16" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1302,7 +1670,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>LNG 탱크 BOR 예측 계산 시트 (정상상태 열전달 모델)</t>
         </is>
@@ -1343,7 +1711,7 @@
           <t>탱크 반지름 r [m]</t>
         </is>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="10">
         <f>Input!B4/2</f>
         <v/>
       </c>
@@ -1352,9 +1720,10 @@
           <t>m</t>
         </is>
       </c>
-      <c r="D4" s="4">
-        <f> 직경 / 2</f>
-        <v/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>직경 / 2</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
@@ -1363,7 +1732,7 @@
           <t>원통부 외면 표면적 [m²]</t>
         </is>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="10">
         <f>2*PI()*B4*Input!B5</f>
         <v/>
       </c>
@@ -1372,9 +1741,10 @@
           <t>m²</t>
         </is>
       </c>
-      <c r="D5" s="4">
-        <f> 2π r L</f>
-        <v/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2π r L</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
@@ -1383,7 +1753,7 @@
           <t>양단 반구 표면적 [m²]</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="10">
         <f>4*PI()*B4^2</f>
         <v/>
       </c>
@@ -1392,9 +1762,10 @@
           <t>m²</t>
         </is>
       </c>
-      <c r="D6" s="4">
-        <f> 4π r²  (양쪽 반구 합)</f>
-        <v/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>4π r²  (양쪽 반구 합)</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
@@ -1403,7 +1774,7 @@
           <t>총 표면적 A [m²]</t>
         </is>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="10">
         <f>B5+B6</f>
         <v/>
       </c>
@@ -1424,7 +1795,7 @@
           <t>탱크 내부 체적 V [m³]</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="10">
         <f>PI()*B4^2*Input!B5+(4/3)*PI()*B4^3</f>
         <v/>
       </c>
@@ -1433,9 +1804,10 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="D8" s="4">
-        <f> π r² L + (4/3)π r³</f>
-        <v/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>π r² L + (4/3)π r³</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
@@ -1444,7 +1816,7 @@
           <t>LNG 체적 V_LNG [m³]</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="10">
         <f>B8*Input!B6/100</f>
         <v/>
       </c>
@@ -1453,9 +1825,10 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="D9" s="4">
-        <f> V_tank × 충전율(%)</f>
-        <v/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>V_tank × 충전율(%)</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1471,8 +1844,8 @@
           <t>단열재 k값 (VLOOKUP) [W/m·K]</t>
         </is>
       </c>
-      <c r="B11" s="12">
-        <f>VLOOKUP(Input!B11,PropertyDB!A4:B9,2,FALSE)</f>
+      <c r="B11" s="10">
+        <f>VLOOKUP(Input!B13,PropertyDB!A4:B9,2,FALSE)</f>
         <v/>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1492,8 +1865,8 @@
           <t>진공보정계수 (고진공 시 keff 감소)</t>
         </is>
       </c>
-      <c r="B12" s="12">
-        <f>IF(Input!B13&lt;10,0.7,IF(Input!B13&lt;100,0.85,1.0))</f>
+      <c r="B12" s="10">
+        <f>IF(Input!B15&lt;10,0.7,IF(Input!B15&lt;100,0.85,1.0))</f>
         <v/>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1513,7 +1886,7 @@
           <t>유효 열전도율 keff [W/m·K]</t>
         </is>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="10">
         <f>B11*B12</f>
         <v/>
       </c>
@@ -1522,9 +1895,10 @@
           <t>W/m·K</t>
         </is>
       </c>
-      <c r="D13" s="4">
-        <f> k × 진공보정계수</f>
-        <v/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>k × 진공보정계수</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
@@ -1533,8 +1907,8 @@
           <t>열저항 R [K/W]</t>
         </is>
       </c>
-      <c r="B14" s="12">
-        <f>Input!B12/(B13*B7)</f>
+      <c r="B14" s="10">
+        <f>Input!B14/(B13*B7)</f>
         <v/>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1542,9 +1916,10 @@
           <t>K/W</t>
         </is>
       </c>
-      <c r="D14" s="4">
-        <f> 두께 / (keff × A)</f>
-        <v/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>두께 / (keff × A)</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -1560,8 +1935,8 @@
           <t>성분1 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B16" s="12">
-        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,3,FALSE)</f>
+      <c r="B16" s="10">
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1581,8 +1956,8 @@
           <t>성분2 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B17" s="12">
-        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,3,FALSE)</f>
+      <c r="B17" s="10">
+        <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1598,8 +1973,8 @@
           <t>성분3 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B18" s="12">
-        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,3,FALSE)</f>
+      <c r="B18" s="10">
+        <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1615,8 +1990,8 @@
           <t>평균 잠열 ΔHvap [kJ/kg]</t>
         </is>
       </c>
-      <c r="B19" s="12">
-        <f>(B16*Input!B22+B17*Input!B23+B18*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
+      <c r="B19" s="10">
+        <f>(B16*Input!B24+B17*Input!B25+B18*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1636,8 +2011,8 @@
           <t>성분1 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B20" s="12">
-        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,4,FALSE)</f>
+      <c r="B20" s="10">
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1653,8 +2028,8 @@
           <t>성분2 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B21" s="12">
-        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,4,FALSE)</f>
+      <c r="B21" s="10">
+        <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1670,8 +2045,8 @@
           <t>성분3 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B22" s="12">
-        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,4,FALSE)</f>
+      <c r="B22" s="10">
+        <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1687,8 +2062,8 @@
           <t>평균 밀도 ρ [kg/m³]</t>
         </is>
       </c>
-      <c r="B23" s="12">
-        <f>(B20*Input!B22+B21*Input!B23+B22*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
+      <c r="B23" s="10">
+        <f>(B20*Input!B24+B21*Input!B25+B22*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1708,8 +2083,8 @@
           <t>성분1 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B24" s="12">
-        <f>VLOOKUP(Input!A22,PropertyDB!A13:E18,5,FALSE)</f>
+      <c r="B24" s="10">
+        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1725,8 +2100,8 @@
           <t>성분2 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B25" s="12">
-        <f>VLOOKUP(Input!A23,PropertyDB!A13:E18,5,FALSE)</f>
+      <c r="B25" s="10">
+        <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1742,8 +2117,8 @@
           <t>성분3 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B26" s="12">
-        <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,5,FALSE)</f>
+      <c r="B26" s="10">
+        <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1759,8 +2134,8 @@
           <t>평균 비등점 T_bp [℃]</t>
         </is>
       </c>
-      <c r="B27" s="12">
-        <f>(B24*Input!B22+B25*Input!B23+B26*Input!B24)/(Input!B22+Input!B23+Input!B24)</f>
+      <c r="B27" s="10">
+        <f>(B24*Input!B24+B25*Input!B25+B26*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1787,8 +2162,8 @@
           <t>압력보정계수</t>
         </is>
       </c>
-      <c r="B29" s="12">
-        <f>MAX(0.8,1-((Input!B8-1.013)*0.05))</f>
+      <c r="B29" s="10">
+        <f>MAX(0.8,1-((Input!B10-1.013)*0.05))</f>
         <v/>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1815,8 +2190,8 @@
           <t>온도차 ΔT [K]</t>
         </is>
       </c>
-      <c r="B31" s="12">
-        <f>Input!B9-B27</f>
+      <c r="B31" s="10">
+        <f>Input!B11-B27</f>
         <v/>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1824,9 +2199,10 @@
           <t>K</t>
         </is>
       </c>
-      <c r="D31" s="4">
-        <f> 외부온도 - LNG 평균비등점</f>
-        <v/>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>외부온도 - LNG 평균비등점</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -1835,7 +2211,7 @@
           <t>탱크 열침투 Q_tank [W]</t>
         </is>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="10">
         <f>B31/B14</f>
         <v/>
       </c>
@@ -1844,9 +2220,10 @@
           <t>W</t>
         </is>
       </c>
-      <c r="D32" s="4">
-        <f> ΔT / R</f>
-        <v/>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>ΔT / R</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -1855,8 +2232,8 @@
           <t>배관 보냉계수 (VLOOKUP)</t>
         </is>
       </c>
-      <c r="B33" s="12">
-        <f>VLOOKUP(Input!B15,PropertyDB!A22:B24,2,FALSE)</f>
+      <c r="B33" s="10">
+        <f>VLOOKUP(Input!B17,PropertyDB!A22:B24,2,FALSE)</f>
         <v/>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1876,8 +2253,8 @@
           <t>배관 열침투 Q_pipe [W]</t>
         </is>
       </c>
-      <c r="B34" s="12">
-        <f>B32*(Input!B16/100)*B33</f>
+      <c r="B34" s="10">
+        <f>B32*(Input!B18/100)*B33</f>
         <v/>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1885,9 +2262,10 @@
           <t>W</t>
         </is>
       </c>
-      <c r="D34" s="4">
-        <f> Q_tank × 배관비율 × 배관계수</f>
-        <v/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Q_tank × 배관비율 × 배관계수</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -1896,7 +2274,7 @@
           <t>총 열침투 Q_total [W]</t>
         </is>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="10">
         <f>B32+B34</f>
         <v/>
       </c>
@@ -1905,9 +2283,10 @@
           <t>W</t>
         </is>
       </c>
-      <c r="D35" s="4">
-        <f> Q_tank + Q_pipe</f>
-        <v/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Q_tank + Q_pipe</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -1923,7 +2302,7 @@
           <t>BOG 질량유량 [kg/s]</t>
         </is>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="10">
         <f>B35/(B19*1000)</f>
         <v/>
       </c>
@@ -1932,9 +2311,10 @@
           <t>kg/s</t>
         </is>
       </c>
-      <c r="D37" s="4">
-        <f> Q_total / ΔHvap[J/kg]</f>
-        <v/>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Q_total / ΔHvap[J/kg]</t>
+        </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
@@ -1943,7 +2323,7 @@
           <t>BOG 일일 증발량 [kg/day]</t>
         </is>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="10">
         <f>B37*86400*B29</f>
         <v/>
       </c>
@@ -1952,9 +2332,10 @@
           <t>kg/day</t>
         </is>
       </c>
-      <c r="D38" s="4">
-        <f> BOG유량 × 86400 × 압력보정</f>
-        <v/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>BOG유량 × 86400 × 압력보정</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
@@ -1963,7 +2344,7 @@
           <t>LNG 총 질량 [kg]</t>
         </is>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="10">
         <f>B9*B23</f>
         <v/>
       </c>
@@ -1972,9 +2353,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="D39" s="4">
-        <f> V_LNG × 평균밀도</f>
-        <v/>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>V_LNG × 평균밀도</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
@@ -1983,7 +2365,7 @@
           <t>★ BOR [%/day]</t>
         </is>
       </c>
-      <c r="B40" s="13">
+      <c r="B40" s="17">
         <f>B38/B39*100</f>
         <v/>
       </c>
@@ -2004,7 +2386,7 @@
           <t>★ BOG [kg/h]</t>
         </is>
       </c>
-      <c r="B41" s="13">
+      <c r="B41" s="17">
         <f>B38/24</f>
         <v/>
       </c>
@@ -2025,7 +2407,7 @@
           <t>★ BOG [kg/day]</t>
         </is>
       </c>
-      <c r="B42" s="13">
+      <c r="B42" s="17">
         <f>B38</f>
         <v/>
       </c>
@@ -2070,7 +2452,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>실측 BOG → BOR 역산 및 예측 비교 (4_계측보정)</t>
         </is>
@@ -2131,8 +2513,8 @@
           <t>계측 시간 [h]</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>Input!B19</f>
+      <c r="B5" s="10">
+        <f>Input!B21</f>
         <v/>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2159,8 +2541,8 @@
           <t>안정화 보정계수</t>
         </is>
       </c>
-      <c r="B7" s="12">
-        <f>IF(Input!B18&lt;6,1.15,IF(Input!B18&lt;12,1.05,1.0))</f>
+      <c r="B7" s="10">
+        <f>IF(Input!B20&lt;6,1.15,IF(Input!B20&lt;12,1.05,1.0))</f>
         <v/>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2180,7 +2562,7 @@
           <t>실측 BOG [kg/h]</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="10">
         <f>B4/B5*B7</f>
         <v/>
       </c>
@@ -2189,9 +2571,10 @@
           <t>kg/h</t>
         </is>
       </c>
-      <c r="D8" s="4">
-        <f> 실측량 / 계측시간 × 보정계수</f>
-        <v/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>실측량 / 계측시간 × 보정계수</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -2200,7 +2583,7 @@
           <t>실측 BOG [kg/day]</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="10">
         <f>B8*24</f>
         <v/>
       </c>
@@ -2209,9 +2592,10 @@
           <t>kg/day</t>
         </is>
       </c>
-      <c r="D9" s="4">
-        <f> 시간당 × 24</f>
-        <v/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>시간당 × 24</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -2220,7 +2604,7 @@
           <t>LNG 총 질량 [kg]</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="10">
         <f>BOR_Calc!B39</f>
         <v/>
       </c>
@@ -2241,7 +2625,7 @@
           <t>★ 실측 BOR [%/day]</t>
         </is>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <f>B9/B10*100</f>
         <v/>
       </c>
@@ -2250,9 +2634,10 @@
           <t>%/day</t>
         </is>
       </c>
-      <c r="D11" s="4">
-        <f> 실측BOG일일 / LNG총질량 × 100</f>
-        <v/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>실측BOG일일 / LNG총질량 × 100</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -2268,7 +2653,7 @@
           <t>★ 예측 BOR [%/day]</t>
         </is>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="17">
         <f>BOR_Calc!B40</f>
         <v/>
       </c>
@@ -2289,7 +2674,7 @@
           <t>오차율 [%]</t>
         </is>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="18">
         <f>(B11-B13)/B13*100</f>
         <v/>
       </c>
@@ -2298,9 +2683,10 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D14" s="4">
-        <f> (실측 - 예측) / 예측 × 100</f>
-        <v/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>(실측 - 예측) / 예측 × 100</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -2309,7 +2695,7 @@
           <t>판정</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="18">
         <f>IF(ABS(B14)&lt;10,"✅ 양호","⚠ 재계측 권장")</f>
         <v/>
       </c>
@@ -2325,7 +2711,7 @@
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>📌 주의: 이 모델은 정상상태(steady-state) 열전달 기반의 설계 예측용 모델입니다.
 실측값과의 오차가 10% 이상이면 단열재 물성, 충전율, 탱크 형상 등 입력값을 재확인하거나

</xml_diff>

<commit_message>
Replace Input cell tank diagram with matplotlib tank drawings
</commit_message>
<xml_diff>
--- a/LNG_BOR_Model.xlsx
+++ b/LNG_BOR_Model.xlsx
@@ -68,7 +68,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -102,11 +102,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4C6E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
@@ -134,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,11 +146,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -180,13 +170,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -263,6 +253,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3143250" cy="3314700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4095750" cy="3009900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -607,7 +652,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>▶ 탱크 형상(고정) 및 사양 정보</t>
+          <t>▶ 탱크 도면 (단열재 층 포함) 및 사양 정보</t>
         </is>
       </c>
     </row>
@@ -646,15 +691,6 @@
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>원통형 LNG 탱크 (고정)</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -675,13 +711,6 @@
           <t>0~100</t>
         </is>
       </c>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -689,7 +718,7 @@
           <t>탱크 내부 체적 [m³]</t>
         </is>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="6">
         <f>PI()*(B4/2)^2*B5+(4/3)*PI()*(B4/2)^3</f>
         <v/>
       </c>
@@ -703,13 +732,6 @@
           <t>내경·길이로 자동 계산</t>
         </is>
       </c>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="8" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -717,7 +739,7 @@
           <t>LNG 체적 [m³]</t>
         </is>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="6">
         <f>B7*B6/100</f>
         <v/>
       </c>
@@ -731,13 +753,6 @@
           <t>체적 × 충전율</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="8" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -745,11 +760,6 @@
           <t>▶ 운전 조건</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -803,7 +813,7 @@
           <t>탱크 내경</t>
         </is>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="7">
         <f>B4</f>
         <v/>
       </c>
@@ -839,7 +849,7 @@
           <t>탱크 길이</t>
         </is>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="7">
         <f>B5</f>
         <v/>
       </c>
@@ -869,7 +879,7 @@
           <t>충전율</t>
         </is>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="7">
         <f>B6</f>
         <v/>
       </c>
@@ -903,7 +913,7 @@
           <t>탱크 내부 체적</t>
         </is>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="7">
         <f>B7</f>
         <v/>
       </c>
@@ -924,7 +934,7 @@
           <t>LNG 체적</t>
         </is>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="7">
         <f>B8</f>
         <v/>
       </c>
@@ -960,7 +970,7 @@
           <t>내부 압력</t>
         </is>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="7">
         <f>B10</f>
         <v/>
       </c>
@@ -994,7 +1004,7 @@
           <t>외부 온도</t>
         </is>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="7">
         <f>B11</f>
         <v/>
       </c>
@@ -1015,7 +1025,7 @@
           <t>단열재 종류</t>
         </is>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="7">
         <f>B13</f>
         <v/>
       </c>
@@ -1049,7 +1059,7 @@
           <t>단열재 두께</t>
         </is>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="7">
         <f>B14</f>
         <v/>
       </c>
@@ -1083,7 +1093,7 @@
           <t>진공도</t>
         </is>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="7">
         <f>B15</f>
         <v/>
       </c>
@@ -1104,7 +1114,7 @@
           <t>배관 보냉/진공</t>
         </is>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="7">
         <f>B17</f>
         <v/>
       </c>
@@ -1115,22 +1125,22 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>성분 이름</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>몰분율 [mol%]</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -1140,7 +1150,7 @@
           <t>배관 열유입 비율</t>
         </is>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="7">
         <f>B18</f>
         <v/>
       </c>
@@ -1174,7 +1184,7 @@
           <t>성분1 이름</t>
         </is>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="7">
         <f>A24</f>
         <v/>
       </c>
@@ -1204,7 +1214,7 @@
           <t>성분1 몰분율</t>
         </is>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="7">
         <f>B24</f>
         <v/>
       </c>
@@ -1238,7 +1248,7 @@
           <t>성분2 이름</t>
         </is>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="7">
         <f>A25</f>
         <v/>
       </c>
@@ -1254,7 +1264,7 @@
           <t>성분2 몰분율</t>
         </is>
       </c>
-      <c r="G27" s="10">
+      <c r="G27" s="7">
         <f>B25</f>
         <v/>
       </c>
@@ -1270,7 +1280,7 @@
           <t>성분3 이름</t>
         </is>
       </c>
-      <c r="G28" s="10">
+      <c r="G28" s="7">
         <f>A26</f>
         <v/>
       </c>
@@ -1286,7 +1296,7 @@
           <t>성분3 몰분율</t>
         </is>
       </c>
-      <c r="G29" s="10">
+      <c r="G29" s="7">
         <f>B26</f>
         <v/>
       </c>
@@ -1297,7 +1307,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A22:D22"/>
@@ -1307,7 +1317,6 @@
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="F11:H11"/>
-    <mergeCell ref="G5:K9"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="입력 오류" error="목록에서 선택하세요" type="list">
@@ -1321,6 +1330,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1342,7 +1352,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>LNG BOR 예측 모델 — 물성 데이터베이스 (2_물성DB)</t>
         </is>
@@ -1356,74 +1366,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>단열재 종류</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>열전도율 k [W/m·K]</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Polyurethane Foam (PUF)</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="11" t="n">
         <v>0.025</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Perlite(대기압)</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="11" t="n">
         <v>0.04</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Perlite(진공)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="11" t="n">
         <v>0.0015</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>MLI(다층진공단열)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="11" t="n">
         <v>0.0005</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Glass Wool</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="11" t="n">
         <v>0.038</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Vacuum Panel</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="11" t="n">
         <v>0.008</v>
       </c>
     </row>
@@ -1435,164 +1445,164 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>분자량
 [g/mol]</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>잠열 ΔHvap
 [kJ/kg]</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>액밀도
 [kg/m³]</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>비등점
 [℃]</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Methane</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="13" t="n">
         <v>16.04</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="13" t="n">
         <v>511</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="13" t="n">
         <v>422.6</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="13" t="n">
         <v>-161.5</v>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>주성분</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Ethane</t>
         </is>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="13" t="n">
         <v>30.07</v>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="13" t="n">
         <v>489</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="13" t="n">
         <v>544.1</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="13" t="n">
         <v>-88.59999999999999</v>
       </c>
-      <c r="F14" s="16" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Propane</t>
         </is>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="13" t="n">
         <v>44.1</v>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="13" t="n">
         <v>426</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="13" t="n">
         <v>581</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="13" t="n">
         <v>-42.1</v>
       </c>
-      <c r="F15" s="16" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Nitrogen</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B16" s="13" t="n">
         <v>28.01</v>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="13" t="n">
         <v>199</v>
       </c>
-      <c r="D16" s="16" t="n">
+      <c r="D16" s="13" t="n">
         <v>806.6</v>
       </c>
-      <c r="E16" s="16" t="n">
+      <c r="E16" s="13" t="n">
         <v>-195.8</v>
       </c>
-      <c r="F16" s="16" t="inlineStr"/>
+      <c r="F16" s="13" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>i-Butane</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B17" s="13" t="n">
         <v>58.12</v>
       </c>
-      <c r="C17" s="16" t="n">
+      <c r="C17" s="13" t="n">
         <v>366</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="13" t="n">
         <v>593.4</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E17" s="13" t="n">
         <v>-11.7</v>
       </c>
-      <c r="F17" s="16" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>n-Butane</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="13" t="n">
         <v>58.12</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="13" t="n">
         <v>385</v>
       </c>
-      <c r="D18" s="16" t="n">
+      <c r="D18" s="13" t="n">
         <v>601.8</v>
       </c>
-      <c r="E18" s="16" t="n">
+      <c r="E18" s="13" t="n">
         <v>-0.5</v>
       </c>
-      <c r="F18" s="16" t="inlineStr"/>
+      <c r="F18" s="13" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1602,44 +1612,44 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>배관 상태</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>열유입 계수</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>보냉없음</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
+      <c r="B22" s="13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>일반보냉</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="13" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>진공배관</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="13" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1670,7 +1680,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>LNG 탱크 BOR 예측 계산 시트 (정상상태 열전달 모델)</t>
         </is>
@@ -1711,7 +1721,7 @@
           <t>탱크 반지름 r [m]</t>
         </is>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <f>Input!B4/2</f>
         <v/>
       </c>
@@ -1732,7 +1742,7 @@
           <t>원통부 외면 표면적 [m²]</t>
         </is>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="7">
         <f>2*PI()*B4*Input!B5</f>
         <v/>
       </c>
@@ -1753,7 +1763,7 @@
           <t>양단 반구 표면적 [m²]</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="7">
         <f>4*PI()*B4^2</f>
         <v/>
       </c>
@@ -1774,7 +1784,7 @@
           <t>총 표면적 A [m²]</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <f>B5+B6</f>
         <v/>
       </c>
@@ -1795,7 +1805,7 @@
           <t>탱크 내부 체적 V [m³]</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <f>PI()*B4^2*Input!B5+(4/3)*PI()*B4^3</f>
         <v/>
       </c>
@@ -1816,7 +1826,7 @@
           <t>LNG 체적 V_LNG [m³]</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="7">
         <f>B8*Input!B6/100</f>
         <v/>
       </c>
@@ -1844,7 +1854,7 @@
           <t>단열재 k값 (VLOOKUP) [W/m·K]</t>
         </is>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="7">
         <f>VLOOKUP(Input!B13,PropertyDB!A4:B9,2,FALSE)</f>
         <v/>
       </c>
@@ -1865,7 +1875,7 @@
           <t>진공보정계수 (고진공 시 keff 감소)</t>
         </is>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="7">
         <f>IF(Input!B15&lt;10,0.7,IF(Input!B15&lt;100,0.85,1.0))</f>
         <v/>
       </c>
@@ -1886,7 +1896,7 @@
           <t>유효 열전도율 keff [W/m·K]</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="7">
         <f>B11*B12</f>
         <v/>
       </c>
@@ -1907,7 +1917,7 @@
           <t>열저항 R [K/W]</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="7">
         <f>Input!B14/(B13*B7)</f>
         <v/>
       </c>
@@ -1935,7 +1945,7 @@
           <t>성분1 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="7">
         <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
@@ -1956,7 +1966,7 @@
           <t>성분2 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="7">
         <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
@@ -1973,7 +1983,7 @@
           <t>성분3 잠열 [kJ/kg]</t>
         </is>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="7">
         <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,3,FALSE)</f>
         <v/>
       </c>
@@ -1990,7 +2000,7 @@
           <t>평균 잠열 ΔHvap [kJ/kg]</t>
         </is>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="7">
         <f>(B16*Input!B24+B17*Input!B25+B18*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
@@ -2011,7 +2021,7 @@
           <t>성분1 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="7">
         <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
@@ -2028,7 +2038,7 @@
           <t>성분2 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="7">
         <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
@@ -2045,7 +2055,7 @@
           <t>성분3 액밀도 [kg/m³]</t>
         </is>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="7">
         <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,4,FALSE)</f>
         <v/>
       </c>
@@ -2062,7 +2072,7 @@
           <t>평균 밀도 ρ [kg/m³]</t>
         </is>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="7">
         <f>(B20*Input!B24+B21*Input!B25+B22*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
@@ -2083,7 +2093,7 @@
           <t>성분1 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="7">
         <f>VLOOKUP(Input!A24,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
@@ -2100,7 +2110,7 @@
           <t>성분2 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="7">
         <f>VLOOKUP(Input!A25,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
@@ -2117,7 +2127,7 @@
           <t>성분3 비등점 [℃]</t>
         </is>
       </c>
-      <c r="B26" s="10">
+      <c r="B26" s="7">
         <f>VLOOKUP(Input!A26,PropertyDB!A13:E18,5,FALSE)</f>
         <v/>
       </c>
@@ -2134,7 +2144,7 @@
           <t>평균 비등점 T_bp [℃]</t>
         </is>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="7">
         <f>(B24*Input!B24+B25*Input!B25+B26*Input!B26)/(Input!B24+Input!B25+Input!B26)</f>
         <v/>
       </c>
@@ -2162,7 +2172,7 @@
           <t>압력보정계수</t>
         </is>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="7">
         <f>MAX(0.8,1-((Input!B10-1.013)*0.05))</f>
         <v/>
       </c>
@@ -2190,7 +2200,7 @@
           <t>온도차 ΔT [K]</t>
         </is>
       </c>
-      <c r="B31" s="10">
+      <c r="B31" s="7">
         <f>Input!B11-B27</f>
         <v/>
       </c>
@@ -2211,7 +2221,7 @@
           <t>탱크 열침투 Q_tank [W]</t>
         </is>
       </c>
-      <c r="B32" s="10">
+      <c r="B32" s="7">
         <f>B31/B14</f>
         <v/>
       </c>
@@ -2232,7 +2242,7 @@
           <t>배관 보냉계수 (VLOOKUP)</t>
         </is>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="7">
         <f>VLOOKUP(Input!B17,PropertyDB!A22:B24,2,FALSE)</f>
         <v/>
       </c>
@@ -2253,7 +2263,7 @@
           <t>배관 열침투 Q_pipe [W]</t>
         </is>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="7">
         <f>B32*(Input!B18/100)*B33</f>
         <v/>
       </c>
@@ -2274,7 +2284,7 @@
           <t>총 열침투 Q_total [W]</t>
         </is>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="7">
         <f>B32+B34</f>
         <v/>
       </c>
@@ -2302,7 +2312,7 @@
           <t>BOG 질량유량 [kg/s]</t>
         </is>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="7">
         <f>B35/(B19*1000)</f>
         <v/>
       </c>
@@ -2323,7 +2333,7 @@
           <t>BOG 일일 증발량 [kg/day]</t>
         </is>
       </c>
-      <c r="B38" s="10">
+      <c r="B38" s="7">
         <f>B37*86400*B29</f>
         <v/>
       </c>
@@ -2344,7 +2354,7 @@
           <t>LNG 총 질량 [kg]</t>
         </is>
       </c>
-      <c r="B39" s="10">
+      <c r="B39" s="7">
         <f>B9*B23</f>
         <v/>
       </c>
@@ -2365,7 +2375,7 @@
           <t>★ BOR [%/day]</t>
         </is>
       </c>
-      <c r="B40" s="17">
+      <c r="B40" s="14">
         <f>B38/B39*100</f>
         <v/>
       </c>
@@ -2386,7 +2396,7 @@
           <t>★ BOG [kg/h]</t>
         </is>
       </c>
-      <c r="B41" s="17">
+      <c r="B41" s="14">
         <f>B38/24</f>
         <v/>
       </c>
@@ -2407,7 +2417,7 @@
           <t>★ BOG [kg/day]</t>
         </is>
       </c>
-      <c r="B42" s="17">
+      <c r="B42" s="14">
         <f>B38</f>
         <v/>
       </c>
@@ -2452,7 +2462,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>실측 BOG → BOR 역산 및 예측 비교 (4_계측보정)</t>
         </is>
@@ -2513,7 +2523,7 @@
           <t>계측 시간 [h]</t>
         </is>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="7">
         <f>Input!B21</f>
         <v/>
       </c>
@@ -2541,7 +2551,7 @@
           <t>안정화 보정계수</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="7">
         <f>IF(Input!B20&lt;6,1.15,IF(Input!B20&lt;12,1.05,1.0))</f>
         <v/>
       </c>
@@ -2562,7 +2572,7 @@
           <t>실측 BOG [kg/h]</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="7">
         <f>B4/B5*B7</f>
         <v/>
       </c>
@@ -2583,7 +2593,7 @@
           <t>실측 BOG [kg/day]</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="7">
         <f>B8*24</f>
         <v/>
       </c>
@@ -2604,7 +2614,7 @@
           <t>LNG 총 질량 [kg]</t>
         </is>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="7">
         <f>BOR_Calc!B39</f>
         <v/>
       </c>
@@ -2625,7 +2635,7 @@
           <t>★ 실측 BOR [%/day]</t>
         </is>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="14">
         <f>B9/B10*100</f>
         <v/>
       </c>
@@ -2653,7 +2663,7 @@
           <t>★ 예측 BOR [%/day]</t>
         </is>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="14">
         <f>BOR_Calc!B40</f>
         <v/>
       </c>
@@ -2674,7 +2684,7 @@
           <t>오차율 [%]</t>
         </is>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="15">
         <f>(B11-B13)/B13*100</f>
         <v/>
       </c>
@@ -2695,7 +2705,7 @@
           <t>판정</t>
         </is>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="15">
         <f>IF(ABS(B14)&lt;10,"✅ 양호","⚠ 재계측 권장")</f>
         <v/>
       </c>
@@ -2711,7 +2721,7 @@
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>📌 주의: 이 모델은 정상상태(steady-state) 열전달 기반의 설계 예측용 모델입니다.
 실측값과의 오차가 10% 이상이면 단열재 물성, 충전율, 탱크 형상 등 입력값을 재확인하거나

</xml_diff>